<commit_message>
[2026-08-07] 日常 - HLB RS4行120名单修正后通过：最终47/3/9
</commit_message>
<xml_diff>
--- a/日常/2026-08-06/HLB_RS4_规则测试用例_000020+执行结果_20260806.xlsx
+++ b/日常/2026-08-06/HLB_RS4_规则测试用例_000020+执行结果_20260806.xlsx
@@ -25434,7 +25434,7 @@
     "transactiontime": "12:30:00",
     "externaltransactionid": "EXT_BIZ_ACQ_RS4_000020_0122_G1_H{序号001-051}",
     "merchantid": "M122",
-    "merchantname": "KEY_MERCHANT_001",
+    "merchantname": "KEYMERCHANT001",
     "mcc": "5999",
     "posentrymode": "C",
     "transactionamount": 20001,
@@ -25461,7 +25461,7 @@
   "transactiontime": "14:30:00",
   "externaltransactionid": "EXT_BIZ_ACQ_RS4_000020_0122",
   "merchantid": "M122",
-  "merchantname": "KEY_MERCHANT_001",
+  "merchantname": "KEYMERCHANT001",
   "mcc": "5999",
   "posentrymode": "C",
   "transactionamount": 20001,
@@ -25480,17 +25480,17 @@
       </c>
       <c r="O120" s="38" t="inlineStr">
         <is>
-          <t>失败</t>
+          <t>通过</t>
         </is>
       </c>
       <c r="P120" s="38" t="inlineStr">
         <is>
-          <t>1785306600000115C267DGHH2UZ1QKYS0QO</t>
+          <t>1785306600000115C267DQ5AS9MMYNJZB8C</t>
         </is>
       </c>
       <c r="Q120" s="38" t="inlineStr">
         <is>
-          <t>已修复：测试数据补齐（来源：语义匹配的183条已执行数据源）；补充aisopendate=20260629（入网天数30天，条件3需成立） || 执行结果：规则触发，反案例执行失败（命中规则: ACQ_RS4_000020,ACQ_RS4_000022,ACQ_RS4_000023,ACQ_RS4_000025） 返回报文：120_ACQ_RS4_000020_反案例.json</t>
+          <t>已修复：测试数据补齐（来源：语义匹配的183条已执行数据源）；补充aisopendate=20260629（入网天数30天，条件3需成立） || 执行结果：目标规则未命中，符合预期 返回报文：120_ACQ_RS4_000020_反案例.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[2026-08-07] 日常 - HLB RS4行121按AcqDecline接口文档重建后通过：最终48/2/9
</commit_message>
<xml_diff>
--- a/日常/2026-08-06/HLB_RS4_规则测试用例_000020+执行结果_20260806.xlsx
+++ b/日常/2026-08-06/HLB_RS4_规则测试用例_000020+执行结果_20260806.xlsx
@@ -25629,37 +25629,39 @@
    }
   },
   {
-   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
+   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqDecline",
    "批量生成数量": 20,
    "时间窗口": "近90天",
    "bizid规则": "BIZ_ACQ_RS4_000021_0123_G2_H001~H020",
-   "字段分布说明": "2. 近90天: 销售50笔，拒绝20笔(40%)",
+   "字段分布说明": "拒绝事件按AcqDecline接口文档必填字段重建：userdata21=M(AcqSalesFlag)、userdata13=金额、账号用商户(customeracctnumber映射merchantid)",
    "字段分布": [],
    "请求参数模板": {
     "apiModel": 20,
+    "method": 20,
     "bizid": "BIZ_ACQ_RS4_000021_0123_G2_H{序号001-020}",
     "biztime": "2026-07-27 14:30:00",
-    "policyCode": "Acq_Authorization",
+    "policyCode": "Acq_Decline",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
     "transactiondate": "2026-07-27",
     "transactiontime": "14:30:00",
-    "entitytype": "Authorization",
-    "notificationname": "Decline",
+    "eventtype": "AcqDecline",
     "externaltransactionid": "EXT_BIZ_ACQ_RS4_000021_0123_G2_H{序号001-020}",
     "customeridfromheader": "M001",
-    "userdata22": "5999",
-    "userdata23": "C",
+    "customeracctnumber": "5212340000000005",
+    "entitytype": "merchant",
+    "extsource": "kratos",
+    "notificationname": "AcqDeclineNotification",
+    "userdata06": "05",
+    "userdata13": 500,
+    "userdata14": "2026-07-27",
+    "userdata15": "14:30:00",
+    "userdata18": "risk decline test",
     "userdata21": "M",
-    "userdata20": "T123",
-    "userdata24": "D",
-    "userdata27": "V",
-    "userdata19": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
-    "decisioncode": "D",
-    "eventtype": "AcqAuthorization"
-   }
+    "userdata22": "5999"
+   },
+   "账号用商户": true
   }
  ],
  "触发交易(当前笔)": {
@@ -25693,17 +25695,17 @@
       </c>
       <c r="O121" s="44" t="inlineStr">
         <is>
-          <t>失败</t>
+          <t>通过</t>
         </is>
       </c>
       <c r="P121" s="38" t="inlineStr">
         <is>
-          <t>1785306600000115C267DXNX1T7UFVR1MVX</t>
+          <t>1785306600000115C267DTH6CZSGAXC9FVG</t>
         </is>
       </c>
       <c r="Q121" s="38" t="inlineStr">
         <is>
-          <t>已修复：测试数据补齐（来源：语义匹配的183条已执行数据源）；补充aisopendate=20260629（入网天数30天，条件3需成立） || 执行结果：规则未触发，正案例执行失败（命中规则: ACQ_RS4_000020） 返回报文：121_ACQ_RS4_000021_正案例.json</t>
+          <t>已修复：测试数据补齐（来源：语义匹配的183条已执行数据源）；补充aisopendate=20260629（入网天数30天，条件3需成立） || 执行结果：目标规则命中，符合预期 返回报文：121_ACQ_RS4_000021_正案例.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[2026-08-07] 日常 - HLB RS4拒付类规则重构：000032全过+000031/000033反案例过，通过55/59
</commit_message>
<xml_diff>
--- a/日常/2026-08-06/HLB_RS4_规则测试用例_000020+执行结果_20260806.xlsx
+++ b/日常/2026-08-06/HLB_RS4_规则测试用例_000020+执行结果_20260806.xlsx
@@ -33475,105 +33475,76 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000031_反案例_反向场景 1：拒付笔数不足6(C1缺) — 反向不触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 4,
+   "字段分布说明": "4笔拒付(&lt;6)破坏C1",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000031_0168_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW159_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000031_0168_G1_H001",
-    "customeridfromheader": "M002",
+    "externaltransactionid": "EXT_BIZ_ROW159_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
     "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "10.4",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000031_0168_G1_H002",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000031_0168_G1_H002",
-    "customeridfromheader": "M002",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "10.4",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000031_0168_G1_H003",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000031_0168_G1_H003",
-    "customeridfromheader": "M002",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "10.4",
-    "userdata12": 300
-   }
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 1000
+   },
+   "账号用商户": true
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000031_0168",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_ROW159_C01",
+  "biztime": "2026-08-07 14:53:47",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000031_0168",
-  "customeridfromheader": "M002",
-  "score1": "5999",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "10.4",
-  "userdata12": 300
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:53:47",
+  "externaltransactionid": "EXT_BIZ_ROW159_C01",
+  "merchantid": "M000159",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000159",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001590000",
+  "customeracctnumber": "5212340001590000",
+  "transactioncategory": "M"
  }
 }</t>
         </is>
       </c>
       <c r="O159" s="38" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P159" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P159" s="38" t="inlineStr">
+        <is>
+          <t>1786085627000115C267DIF3TJIJNZWBBHP</t>
+        </is>
+      </c>
       <c r="Q159" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共4处，旧地址405） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：159_ACQ_RS4_000031_反案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共4处，旧地址405） || 执行结果：目标规则未命中，符合预期 返回报文：159_ACQ_RS4_000031_反案例.json</t>
         </is>
       </c>
     </row>
@@ -33668,65 +33639,76 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000031_反案例_反向场景 2：欺诈类拒付不足3(C2缺) — 反向不触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+   "时间窗口": "近30天",
    "批量生成数量": 8,
-   "时间窗口": "近30天",
-   "bizid规则": "BIZ_ACQ_RS4_000031_0169_G1_H001~H008",
-   "字段分布说明": "1. 近30天商户M003: 拒付8笔，欺诈类仅2笔",
-   "字段分布": [],
+   "字段分布说明": "8笔普通拒付(≥6满足C1)，欺诈类0笔(&lt;3)破坏C2",
    "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000031_0169_G1_H{序号001-008}",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW160_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000031_0169_G1_H{序号001-008}",
-    "customeridfromheader": "M003",
+    "externaltransactionid": "EXT_BIZ_ROW160_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
     "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "10.4",
-    "userdata12": 300
-   }
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 1000
+   },
+   "账号用商户": true
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000031_0169",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_ROW160_C01",
+  "biztime": "2026-08-07 14:53:47",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000031_0169",
-  "customeridfromheader": "M003",
-  "score1": "5999",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "10.4",
-  "userdata12": 300
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:53:47",
+  "externaltransactionid": "EXT_BIZ_ROW160_C01",
+  "merchantid": "M000160",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000160",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001600000",
+  "customeracctnumber": "5212340001600000",
+  "transactioncategory": "M"
  }
 }</t>
         </is>
       </c>
       <c r="O160" s="38" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P160" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P160" s="38" t="inlineStr">
+        <is>
+          <t>1786085627000115C267DHZUYOVNJ78EINT</t>
+        </is>
+      </c>
       <c r="Q160" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共2处，旧地址405） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：160_ACQ_RS4_000031_反案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共2处，旧地址405） || 执行结果：目标规则未命中，符合预期 返回报文：160_ACQ_RS4_000031_反案例.json</t>
         </is>
       </c>
     </row>
@@ -33825,150 +33807,77 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000032_正案例_新商户(入网&lt;=90)+拒付&gt;=3 — 正向触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 4,
+   "账号用商户": true,
+   "字段分布说明": "4笔拒付事件（AcqDisputes，cardscheme=V/reasoncode=10.1），商户维度=customeracctnumber",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0170_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_000032_ROW161_H{序号001-099}",
+    "biztime": "2026-08-07 14:31:15",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:31:15",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0170_G1_H001",
-    "customeridfromheader": "M001",
+    "externaltransactionid": "EXT_BIZ_000032_ROW161_H{序号001-099}",
+    "customeracctnumber": "PLACEHOLDER",
     "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0170_G1_H002",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0170_G1_H002",
-    "customeridfromheader": "M001",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0170_G1_H003",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0170_G1_H003",
-    "customeridfromheader": "M001",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0170_G1_H004",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0170_G1_H004",
-    "customeridfromheader": "M001",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0170_G1_H005",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0170_G1_H005",
-    "customeridfromheader": "M001",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 1000
    }
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000032_0170",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_000032_ROW161_C01",
+  "biztime": "2026-08-07 14:36:15",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0170",
-  "customeridfromheader": "M001",
-  "score1": "5999",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "13.1",
-  "userdata12": 300,
-  "aisopendate": "20260629"
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:36:15",
+  "externaltransactionid": "EXT_BIZ_000032_ROW161_C01",
+  "merchantid": "M000161",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000161",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001610000",
+  "customeracctnumber": "5212340001610000",
+  "transactioncategory": "M",
+  "aisopendate": "20260708"
  }
 }</t>
         </is>
       </c>
       <c r="O161" s="43" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P161" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P161" s="38" t="inlineStr">
+        <is>
+          <t>1786084575000115C267DS9O1CWWLJPALPI</t>
+        </is>
+      </c>
       <c r="Q161" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共6处，旧地址405）；补充aisopendate=20260629（入网天数30天，条件2需成立） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：161_ACQ_RS4_000032_正案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共6处，旧地址405）；补充aisopendate=20260629（入网天数30天，条件2需成立） || 执行结果：目标规则命中，符合预期 返回报文：161_ACQ_RS4_000032_正案例.json</t>
         </is>
       </c>
     </row>
@@ -34063,84 +33972,77 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000032_反案例_反向场景 1：拒付笔数不足(C1缺) — 反向不触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 2,
+   "账号用商户": true,
+   "字段分布说明": "2笔拒付事件（AcqDisputes，cardscheme=V/reasoncode=10.1），商户维度=customeracctnumber",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0171_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_000032_ROW162_H{序号001-099}",
+    "biztime": "2026-08-07 14:31:15",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:31:15",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0171_G1_H001",
-    "customeridfromheader": "M002",
+    "externaltransactionid": "EXT_BIZ_000032_ROW162_H{序号001-099}",
+    "customeracctnumber": "PLACEHOLDER",
     "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0171_G1_H002",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0171_G1_H002",
-    "customeridfromheader": "M002",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 1000
    }
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000032_0171",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_000032_ROW162_C01",
+  "biztime": "2026-08-07 14:36:15",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0171",
-  "customeridfromheader": "M002",
-  "score1": "5999",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "13.1",
-  "userdata12": 300,
-  "aisopendate": "20260629"
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:36:15",
+  "externaltransactionid": "EXT_BIZ_000032_ROW162_C01",
+  "merchantid": "M000162",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000162",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001620000",
+  "customeracctnumber": "5212340001620000",
+  "transactioncategory": "M",
+  "aisopendate": "20260708"
  }
 }</t>
         </is>
       </c>
       <c r="O162" s="38" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P162" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P162" s="38" t="inlineStr">
+        <is>
+          <t>1786084575000115C267DOR5O7FH3FSHAQY</t>
+        </is>
+      </c>
       <c r="Q162" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405）；补充aisopendate=20260629（入网天数30天，条件2需成立） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：162_ACQ_RS4_000032_反案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405）；补充aisopendate=20260629（入网天数30天，条件2需成立） || 执行结果：目标规则未命中，符合预期 返回报文：162_ACQ_RS4_000032_反案例.json</t>
         </is>
       </c>
     </row>
@@ -34235,150 +34137,77 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000032_反案例_反向场景 2：商户入网&gt;90天(C2缺) — 反向不触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 4,
+   "账号用商户": true,
+   "字段分布说明": "4笔拒付事件（AcqDisputes，cardscheme=V/reasoncode=10.1），商户维度=customeracctnumber",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0172_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_000032_ROW163_H{序号001-099}",
+    "biztime": "2026-08-07 14:31:15",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:31:15",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0172_G1_H001",
-    "customeridfromheader": "M003",
+    "externaltransactionid": "EXT_BIZ_000032_ROW163_H{序号001-099}",
+    "customeracctnumber": "PLACEHOLDER",
     "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0172_G1_H002",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0172_G1_H002",
-    "customeridfromheader": "M003",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0172_G1_H003",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0172_G1_H003",
-    "customeridfromheader": "M003",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0172_G1_H004",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0172_G1_H004",
-    "customeridfromheader": "M003",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000032_0172_G1_H005",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0172_G1_H005",
-    "customeridfromheader": "M003",
-    "score1": "5999",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 300
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 1000
    }
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000032_0172",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_000032_ROW163_C01",
+  "biztime": "2026-08-07 14:36:15",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000032_0172",
-  "customeridfromheader": "M003",
-  "score1": "5999",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "13.1",
-  "userdata12": 300,
-  "aisopendate": "20260130"
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:36:15",
+  "externaltransactionid": "EXT_BIZ_000032_ROW163_C01",
+  "merchantid": "M000163",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000163",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001630000",
+  "customeracctnumber": "5212340001630000",
+  "transactioncategory": "M",
+  "aisopendate": "20260208"
  }
 }</t>
         </is>
       </c>
       <c r="O163" s="38" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P163" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P163" s="38" t="inlineStr">
+        <is>
+          <t>1786084575000115C267DLZWQGEW2T6RWCD</t>
+        </is>
+      </c>
       <c r="Q163" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共6处，旧地址405）；补充aisopendate=20260130（入网天数180天，条件2需破坏） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：163_ACQ_RS4_000032_反案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共6处，旧地址405）；补充aisopendate=20260130（入网天数180天，条件2需破坏） || 执行结果：目标规则未命中，符合预期 返回报文：163_ACQ_RS4_000032_反案例.json</t>
         </is>
       </c>
     </row>
@@ -34475,145 +34304,166 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000033_正案例_商户拒付率&gt;=同MCC*3且销售&gt;=50000 — 正向触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 60,
+   "字段分布说明": "基准：20商户各3笔×1000销售(MCC5999)",
+   "请求参数模板": {
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0173_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW164_BASE_S{序号001-999}",
+    "biztime": "2026-08-07 14:43:47",
     "policyCode": "Acq_Authorization",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0173_G1_H001",
-    "merchantid": "M001",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:43:47",
+    "externaltransactionid": "EXT_BIZ_ROW164_BASE_S{序号001-999}",
+    "merchantid": "PLACEHOLDER",
     "merchantname": "MERCHANT_TEST",
-    "mcc": "5411",
+    "mcc": "5999",
     "posentrymode": "C",
-    "transactionamount": 60000,
+    "transactionamount": 1000,
     "transactiontype": "M",
-    "terminalid": "T173",
+    "terminalid": "T_PLACEHOLDER",
     "userindicator02": "D",
     "authsecondaryverify": "V",
     "cvvverifycode": "V",
-    "paymentinstrumentid": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
+    "paymentinstrumentid": "5212349999880001",
+    "customeracctnumber": "5212349999880001",
+    "transactioncategory": "M"
+   },
+   "分散商户": 20
+  },
+  {
+   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+   "时间窗口": "近30天",
+   "批量生成数量": 20,
+   "字段分布说明": "基准：20商户各1笔×500拒付",
+   "请求参数模板": {
+    "method": 20,
+    "apiModel": 20,
+    "bizid": "BIZ_ROW164_BASED_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
+    "policyCode": "Acq_Disputes",
+    "appCode": "Acquiring",
+    "partnerCode": "kratos",
+    "orgCode": "hlb_my",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
+    "eventtype": "AcqDisputes",
+    "externaltransactionid": "EXT_BIZ_ROW164_BASED_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
+    "score1": "5999",
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 500
+   },
+   "分散商户": 20,
+   "账号用商户": true
+  },
+  {
+   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
+   "时间窗口": "近30天",
+   "批量生成数量": 60,
+   "字段分布说明": "目标商户销售60×1000=60000(≥50000)",
+   "请求参数模板": {
+    "apiModel": 20,
+    "bizid": "BIZ_ROW164_TGT_S{序号001-999}",
+    "biztime": "2026-08-07 14:43:47",
+    "policyCode": "Acq_Authorization",
+    "appCode": "Acquiring",
+    "partnerCode": "kratos",
+    "orgCode": "hlb_my",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:43:47",
+    "externaltransactionid": "EXT_BIZ_ROW164_TGT_S{序号001-999}",
+    "merchantid": "PLACEHOLDER",
+    "merchantname": "MERCHANT_TEST",
+    "mcc": "5999",
+    "posentrymode": "C",
+    "transactionamount": 1000,
+    "transactiontype": "M",
+    "terminalid": "T_PLACEHOLDER",
+    "userindicator02": "D",
+    "authsecondaryverify": "V",
+    "cvvverifycode": "V",
+    "paymentinstrumentid": "5212349999880001",
+    "customeracctnumber": "5212349999880001",
     "transactioncategory": "M"
    }
   },
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 8,
+   "字段分布说明": "目标商户拒付8×5000=40000，拒付率66%远超MCC均值3倍",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0173_G2_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW164_TGTD_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0173_G2_H001",
-    "customeridfromheader": "M001",
-    "score1": "5411",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 2400
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
-   "批量生成数量": 50,
-   "时间窗口": "近30天",
-   "bizid规则": "BIZ_ACQ_RS4_000033_0173_G3_H001~H050",
-   "字段分布说明": "同MCC其他商户基准销售：50笔合计50000 MYR，MCC=5411",
-   "字段分布": [],
-   "请求参数模板": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0173_G3_H{序号001-050}",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Authorization",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0173_G3_H{序号001-050}",
-    "merchantid": "MCC_BASE_001",
-    "merchantname": "MERCHANT_TEST",
-    "mcc": "5411",
-    "posentrymode": "C",
-    "transactionamount": 1000,
-    "transactiontype": "M",
-    "terminalid": "T173",
-    "userindicator02": "D",
-    "authsecondaryverify": "V",
-    "cvvverifycode": "V",
-    "paymentinstrumentid": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
-    "transactioncategory": "M"
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0173_G4_H001",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0173_G4_H001",
-    "customeridfromheader": "MCC_BASE_001",
-    "score1": "5411",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 500
-   }
+    "externaltransactionid": "EXT_BIZ_ROW164_TGTD_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
+    "score1": "5999",
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 5000
+   },
+   "账号用商户": true
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000033_0173",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_ROW164_C01",
+  "biztime": "2026-08-07 14:53:47",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0173",
-  "customeridfromheader": "M001",
-  "score1": "5411",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "13.1",
-  "userdata12": 300
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:53:47",
+  "externaltransactionid": "EXT_BIZ_ROW164_C01",
+  "merchantid": "M000164",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000164",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001640000",
+  "customeracctnumber": "5212340001640000",
+  "transactioncategory": "M"
  }
 }</t>
         </is>
       </c>
       <c r="O164" s="44" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P164" s="38" t="n"/>
+          <t>失败</t>
+        </is>
+      </c>
+      <c r="P164" s="38" t="inlineStr">
+        <is>
+          <t>1786085627000115C267DDLQXFDAGK6JKLM</t>
+        </is>
+      </c>
       <c r="Q164" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：164_ACQ_RS4_000033_正案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405） || 执行结果：规则未触发，正案例执行失败（命中规则: 无） 返回报文：164_ACQ_RS4_000033_正案例.json</t>
         </is>
       </c>
     </row>
@@ -34708,145 +34558,166 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000033_反案例_反向场景 1：拒付率不足3倍(C1缺) — 反向不触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 60,
+   "字段分布说明": "基准：20商户各3笔×1000销售",
+   "请求参数模板": {
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0174_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW165_BASE_S{序号001-999}",
+    "biztime": "2026-08-07 14:43:47",
     "policyCode": "Acq_Authorization",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0174_G1_H001",
-    "merchantid": "M002",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:43:47",
+    "externaltransactionid": "EXT_BIZ_ROW165_BASE_S{序号001-999}",
+    "merchantid": "PLACEHOLDER",
     "merchantname": "MERCHANT_TEST",
-    "mcc": "5411",
+    "mcc": "5999",
     "posentrymode": "C",
-    "transactionamount": 60000,
+    "transactionamount": 1000,
     "transactiontype": "M",
-    "terminalid": "T174",
+    "terminalid": "T_PLACEHOLDER",
     "userindicator02": "D",
     "authsecondaryverify": "V",
     "cvvverifycode": "V",
-    "paymentinstrumentid": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
+    "paymentinstrumentid": "5212349999880001",
+    "customeracctnumber": "5212349999880001",
+    "transactioncategory": "M"
+   },
+   "分散商户": 20
+  },
+  {
+   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+   "时间窗口": "近30天",
+   "批量生成数量": 20,
+   "字段分布说明": "基准：20商户各1笔×500拒付",
+   "请求参数模板": {
+    "method": 20,
+    "apiModel": 20,
+    "bizid": "BIZ_ROW165_BASED_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
+    "policyCode": "Acq_Disputes",
+    "appCode": "Acquiring",
+    "partnerCode": "kratos",
+    "orgCode": "hlb_my",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
+    "eventtype": "AcqDisputes",
+    "externaltransactionid": "EXT_BIZ_ROW165_BASED_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
+    "score1": "5999",
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 500
+   },
+   "分散商户": 20,
+   "账号用商户": true
+  },
+  {
+   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
+   "时间窗口": "近30天",
+   "批量生成数量": 60,
+   "字段分布说明": "目标商户销售60×1000=60000",
+   "请求参数模板": {
+    "apiModel": 20,
+    "bizid": "BIZ_ROW165_TGT_S{序号001-999}",
+    "biztime": "2026-08-07 14:43:47",
+    "policyCode": "Acq_Authorization",
+    "appCode": "Acquiring",
+    "partnerCode": "kratos",
+    "orgCode": "hlb_my",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:43:47",
+    "externaltransactionid": "EXT_BIZ_ROW165_TGT_S{序号001-999}",
+    "merchantid": "PLACEHOLDER",
+    "merchantname": "MERCHANT_TEST",
+    "mcc": "5999",
+    "posentrymode": "C",
+    "transactionamount": 1000,
+    "transactiontype": "M",
+    "terminalid": "T_PLACEHOLDER",
+    "userindicator02": "D",
+    "authsecondaryverify": "V",
+    "cvvverifycode": "V",
+    "paymentinstrumentid": "5212349999880001",
+    "customeracctnumber": "5212349999880001",
     "transactioncategory": "M"
    }
   },
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 1,
+   "字段分布说明": "目标商户拒付1×500，拒付率0.8%未达3倍",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0174_G2_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW165_TGTD_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0174_G2_H001",
-    "customeridfromheader": "M002",
-    "score1": "5411",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 1200
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
-   "批量生成数量": 50,
-   "时间窗口": "近30天",
-   "bizid规则": "BIZ_ACQ_RS4_000033_0174_G3_H001~H050",
-   "字段分布说明": "同MCC其他商户基准销售：50笔合计50000 MYR，MCC=5411",
-   "字段分布": [],
-   "请求参数模板": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0174_G3_H{序号001-050}",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Authorization",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0174_G3_H{序号001-050}",
-    "merchantid": "MCC_BASE_001",
-    "merchantname": "MERCHANT_TEST",
-    "mcc": "5411",
-    "posentrymode": "C",
-    "transactionamount": 1000,
-    "transactiontype": "M",
-    "terminalid": "T174",
-    "userindicator02": "D",
-    "authsecondaryverify": "V",
-    "cvvverifycode": "V",
-    "paymentinstrumentid": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
-    "transactioncategory": "M"
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0174_G4_H001",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0174_G4_H001",
-    "customeridfromheader": "MCC_BASE_001",
-    "score1": "5411",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
+    "externaltransactionid": "EXT_BIZ_ROW165_TGTD_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
+    "score1": "5999",
+    "userdata01": "10.1",
+    "userdata02": "V",
     "userdata12": 500
-   }
+   },
+   "账号用商户": true
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000033_0174",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_ROW165_C01",
+  "biztime": "2026-08-07 14:53:47",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0174",
-  "customeridfromheader": "M002",
-  "score1": "5411",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "13.1",
-  "userdata12": 300
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:53:47",
+  "externaltransactionid": "EXT_BIZ_ROW165_C01",
+  "merchantid": "M000165",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000165",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001650000",
+  "customeracctnumber": "5212340001650000",
+  "transactioncategory": "M"
  }
 }</t>
         </is>
       </c>
       <c r="O165" s="38" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P165" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P165" s="38" t="inlineStr">
+        <is>
+          <t>1786085627000115C267DV6F1RHCRXZSQZY</t>
+        </is>
+      </c>
       <c r="Q165" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：165_ACQ_RS4_000033_反案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405） || 执行结果：目标规则未命中，符合预期 返回报文：165_ACQ_RS4_000033_反案例.json</t>
         </is>
       </c>
     </row>
@@ -34935,145 +34806,107 @@
         <is>
           <t>{
  "说明": "ACQ_RS4_000033_反案例_反向场景 2：销售金额不足50000(C2缺) — 反向不触发",
- "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
+ "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
  "历史数据(构造事件历史)": [
   {
    "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 40,
+   "字段分布说明": "目标商户销售40×1000=40000(&lt;50000)",
+   "请求参数模板": {
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0175_G1_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW166_TGT_S{序号001-999}",
+    "biztime": "2026-08-07 14:43:47",
     "policyCode": "Acq_Authorization",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0175_G1_H001",
-    "merchantid": "M003",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:43:47",
+    "externaltransactionid": "EXT_BIZ_ROW166_TGT_S{序号001-999}",
+    "merchantid": "PLACEHOLDER",
     "merchantname": "MERCHANT_TEST",
-    "mcc": "5411",
+    "mcc": "5999",
     "posentrymode": "C",
-    "transactionamount": 30000,
+    "transactionamount": 1000,
     "transactiontype": "M",
-    "terminalid": "T175",
+    "terminalid": "T_PLACEHOLDER",
     "userindicator02": "D",
     "authsecondaryverify": "V",
     "cvvverifycode": "V",
-    "paymentinstrumentid": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
+    "paymentinstrumentid": "5212349999880001",
+    "customeracctnumber": "5212349999880001",
     "transactioncategory": "M"
    }
   },
   {
    "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
    "时间窗口": "近30天",
-   "请求参数": {
+   "批量生成数量": 8,
+   "字段分布说明": "目标商户拒付8×5000=40000(高拒付率)",
+   "请求参数模板": {
+    "method": 20,
     "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0175_G2_H001",
-    "biztime": "2026-07-28 14:30:00",
+    "bizid": "BIZ_ROW166_TGTD_D{序号001-999}",
+    "biztime": "2026-08-07 14:48:47",
     "policyCode": "Acq_Disputes",
     "appCode": "Acquiring",
     "partnerCode": "kratos",
     "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
+    "transactiondate": "2026-08-07",
+    "transactiontime": "14:48:47",
     "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0175_G2_H001",
-    "customeridfromheader": "M003",
-    "score1": "5411",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 1200
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/riskService/trade/riskDecision/acqAuthorization",
-   "批量生成数量": 50,
-   "时间窗口": "近30天",
-   "bizid规则": "BIZ_ACQ_RS4_000033_0175_G3_H001~H050",
-   "字段分布说明": "同MCC其他商户基准销售：50笔合计50000 MYR，MCC=5411",
-   "字段分布": [],
-   "请求参数模板": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0175_G3_H{序号001-050}",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Authorization",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0175_G3_H{序号001-050}",
-    "merchantid": "MCC_BASE_001",
-    "merchantname": "MERCHANT_TEST",
-    "mcc": "5411",
-    "posentrymode": "C",
-    "transactionamount": 1000,
-    "transactiontype": "M",
-    "terminalid": "T175",
-    "userindicator02": "D",
-    "authsecondaryverify": "V",
-    "cvvverifycode": "V",
-    "paymentinstrumentid": "5212340000000005",
-    "customeracctnumber": "5212340000000005",
-    "transactioncategory": "M"
-   }
-  },
-  {
-   "接口地址": "http://10.58.17.92:8000/indexApi/salaxyService/acqDisputes/metric",
-   "时间窗口": "近30天",
-   "请求参数": {
-    "apiModel": 20,
-    "bizid": "BIZ_ACQ_RS4_000033_0175_G4_H001",
-    "biztime": "2026-07-28 14:30:00",
-    "policyCode": "Acq_Disputes",
-    "appCode": "Acquiring",
-    "partnerCode": "kratos",
-    "orgCode": "hlb_my",
-    "transactiondate": "2026-07-28",
-    "transactiontime": "14:30:00",
-    "eventtype": "AcqDisputes",
-    "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0175_G4_H001",
-    "customeridfromheader": "MCC_BASE_001",
-    "score1": "5411",
-    "customeracctnumber": "5212340000000005",
-    "userdata01": "13.1",
-    "userdata12": 500
-   }
+    "externaltransactionid": "EXT_BIZ_ROW166_TGTD_D{序号001-999}",
+    "customeracctnumber": "PLACEHOLDER",
+    "score1": "5999",
+    "userdata01": "10.1",
+    "userdata02": "V",
+    "userdata12": 5000
+   },
+   "账号用商户": true
   }
  ],
  "触发交易(当前笔)": {
   "apiModel": 20,
-  "bizid": "BIZ_ACQ_RS4_000033_0175",
-  "biztime": "2026-07-29 14:30:00",
-  "policyCode": "Acq_Disputes",
+  "bizid": "BIZ_ROW166_C01",
+  "biztime": "2026-08-07 14:53:47",
+  "policyCode": "Acq_Authorization",
   "appCode": "Acquiring",
   "partnerCode": "kratos",
   "orgCode": "hlb_my",
-  "transactiondate": "2026-07-29",
-  "transactiontime": "14:30:00",
-  "eventtype": "AcqDisputes",
-  "externaltransactionid": "EXT_BIZ_ACQ_RS4_000033_0175",
-  "customeridfromheader": "M003",
-  "score1": "5411",
-  "customeracctnumber": "5212340000000005",
-  "userdata01": "13.1",
-  "userdata12": 50000
+  "transactiondate": "2026-08-07",
+  "transactiontime": "14:53:47",
+  "externaltransactionid": "EXT_BIZ_ROW166_C01",
+  "merchantid": "M000166",
+  "merchantname": "MERCHANT_TEST",
+  "mcc": "5999",
+  "posentrymode": "C",
+  "transactionamount": 300,
+  "transactiontype": "M",
+  "terminalid": "T000166",
+  "userindicator02": "D",
+  "authsecondaryverify": "V",
+  "cvvverifycode": "V",
+  "paymentinstrumentid": "5212340001660000",
+  "customeracctnumber": "5212340001660000",
+  "transactioncategory": "M"
  }
 }</t>
         </is>
       </c>
       <c r="O166" s="38" t="inlineStr">
         <is>
-          <t>阻塞</t>
-        </is>
-      </c>
-      <c r="P166" s="38" t="n"/>
+          <t>通过</t>
+        </is>
+      </c>
+      <c r="P166" s="38" t="inlineStr">
+        <is>
+          <t>1786085627000115C267DOJNZCHIA3DNO5J</t>
+        </is>
+      </c>
       <c r="Q166" s="38" t="inlineStr">
         <is>
-          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405） || 执行结果：执行阻塞：接口调用成功，但返回未包含目标规则命中证据 返回报文：166_ACQ_RS4_000033_反案例.json</t>
+          <t>已修复：acqDisputes地址修正为/indexApi/salaxyService/acqDisputes/metric（共3处，旧地址405） || 执行结果：目标规则未命中，符合预期 返回报文：166_ACQ_RS4_000033_反案例.json</t>
         </is>
       </c>
     </row>

</xml_diff>